<commit_message>
Aktualizacja plikow - 2026-08-31 01:54
</commit_message>
<xml_diff>
--- a/NeuroHeart_Baza_Zasad_Finalna.xlsx
+++ b/NeuroHeart_Baza_Zasad_Finalna.xlsx
@@ -11633,7 +11633,7 @@
       </c>
       <c r="G6" s="36" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H6" s="38" t="n">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="G7" s="36" t="inlineStr">
         <is>
-          <t>d8</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H7" s="38" t="n">
@@ -12205,7 +12205,7 @@
       </c>
       <c r="G13" s="36" t="inlineStr">
         <is>
-          <t>d12+1</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="H13" s="38" t="n">
@@ -12366,7 +12366,7 @@
       </c>
       <c r="G15" s="36" t="inlineStr">
         <is>
-          <t>d12+3</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="H15" s="38" t="n">
@@ -12612,7 +12612,7 @@
       </c>
       <c r="G18" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="H18" s="38" t="n">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="G19" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="H19" s="38" t="n">
@@ -12849,7 +12849,7 @@
       </c>
       <c r="G21" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H21" s="38" t="n">
@@ -13166,12 +13166,12 @@
       </c>
       <c r="F25" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G25" s="36" t="inlineStr">
         <is>
-          <t>d8+2</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="H25" s="38" t="n">
@@ -13249,12 +13249,12 @@
       </c>
       <c r="F26" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G26" s="36" t="inlineStr">
         <is>
-          <t>d12+2</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="H26" s="38" t="n">
@@ -13583,12 +13583,12 @@
       </c>
       <c r="F5" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G5" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="H5" s="36" t="inlineStr">
@@ -13643,7 +13643,7 @@
       </c>
       <c r="AJ5" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>1k8 kłute</t>
         </is>
       </c>
       <c r="AK5" s="43" t="n">
@@ -13683,7 +13683,7 @@
       </c>
       <c r="F6" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G6" s="36" t="inlineStr">
@@ -13740,7 +13740,7 @@
       </c>
       <c r="AJ6" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK6" s="43" t="n">
@@ -13780,12 +13780,12 @@
       </c>
       <c r="F7" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G7" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="H7" s="36" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="AJ7" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>1k10 kłute</t>
         </is>
       </c>
       <c r="AK7" s="43" t="n">
@@ -13883,12 +13883,12 @@
       </c>
       <c r="F8" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G8" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="H8" s="36" t="inlineStr">
@@ -13943,7 +13943,7 @@
       </c>
       <c r="AJ8" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>1k10 kłute</t>
         </is>
       </c>
       <c r="AK8" s="43" t="n">
@@ -13986,12 +13986,12 @@
       </c>
       <c r="F9" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G9" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H9" s="36" t="inlineStr">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="AJ9" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK9" s="43" t="n">
@@ -14086,12 +14086,12 @@
       </c>
       <c r="F10" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G10" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H10" s="36" t="inlineStr">
@@ -14143,7 +14143,7 @@
       </c>
       <c r="AJ10" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK10" s="43" t="n">
@@ -14183,12 +14183,12 @@
       </c>
       <c r="F11" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G11" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H11" s="36" t="inlineStr">
@@ -14240,7 +14240,7 @@
       </c>
       <c r="AJ11" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK11" s="43" t="n">
@@ -14280,12 +14280,12 @@
       </c>
       <c r="F12" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G12" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H12" s="36" t="inlineStr">
@@ -14337,7 +14337,7 @@
       </c>
       <c r="AJ12" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK12" s="43" t="n">
@@ -14377,12 +14377,12 @@
       </c>
       <c r="F13" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G13" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H13" s="36" t="inlineStr">
@@ -14434,7 +14434,7 @@
       </c>
       <c r="AJ13" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK13" s="43" t="n">
@@ -14474,12 +14474,12 @@
       </c>
       <c r="F14" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G14" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H14" s="36" t="inlineStr">
@@ -14531,7 +14531,7 @@
       </c>
       <c r="AJ14" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK14" s="43" t="n">
@@ -14574,12 +14574,12 @@
       </c>
       <c r="F15" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G15" s="36" t="inlineStr">
         <is>
-          <t>d8+1</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="H15" s="36" t="inlineStr">
@@ -14631,7 +14631,7 @@
       </c>
       <c r="AJ15" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k8 kłute</t>
         </is>
       </c>
       <c r="AK15" s="43" t="n">
@@ -14671,12 +14671,12 @@
       </c>
       <c r="F16" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G16" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H16" s="36" t="inlineStr">
@@ -14728,7 +14728,7 @@
       </c>
       <c r="AJ16" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK16" s="43" t="n">
@@ -14774,12 +14774,12 @@
       </c>
       <c r="F17" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G17" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H17" s="36" t="inlineStr">
@@ -14831,7 +14831,7 @@
       </c>
       <c r="AJ17" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK17" s="43" t="n">
@@ -14877,12 +14877,12 @@
       </c>
       <c r="F18" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G18" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="H18" s="36" t="inlineStr">
@@ -14934,7 +14934,7 @@
       </c>
       <c r="AJ18" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k8 kłute</t>
         </is>
       </c>
       <c r="AK18" s="43" t="n">
@@ -14980,12 +14980,12 @@
       </c>
       <c r="F19" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G19" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H19" s="36" t="inlineStr">
@@ -15037,7 +15037,7 @@
       </c>
       <c r="AJ19" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK19" s="43" t="n">
@@ -15083,12 +15083,12 @@
       </c>
       <c r="F20" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G20" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="H20" s="36" t="inlineStr">
@@ -15140,7 +15140,7 @@
       </c>
       <c r="AJ20" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k6 kłute</t>
         </is>
       </c>
       <c r="AK20" s="43" t="n">
@@ -15186,12 +15186,12 @@
       </c>
       <c r="F21" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G21" s="36" t="inlineStr">
         <is>
-          <t>d8+1</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="H21" s="36" t="inlineStr">
@@ -15243,7 +15243,7 @@
       </c>
       <c r="AJ21" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k8 kłute</t>
         </is>
       </c>
       <c r="AK21" s="43" t="n">
@@ -15289,12 +15289,12 @@
       </c>
       <c r="F22" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G22" s="36" t="inlineStr">
         <is>
-          <t>d6+1</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="H22" s="36" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="AJ22" s="41" t="inlineStr">
         <is>
-          <t>Lekkie</t>
+          <t>1k12 kłute</t>
         </is>
       </c>
       <c r="AK22" s="43" t="n">
@@ -15389,12 +15389,12 @@
       </c>
       <c r="F23" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G23" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H23" s="36" t="inlineStr">
@@ -15446,7 +15446,7 @@
       </c>
       <c r="AJ23" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK23" s="43" t="n">
@@ -15489,12 +15489,12 @@
       </c>
       <c r="F24" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G24" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H24" s="36" t="inlineStr">
@@ -15546,7 +15546,7 @@
       </c>
       <c r="AJ24" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK24" s="43" t="n">
@@ -15589,12 +15589,12 @@
       </c>
       <c r="F25" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G25" s="36" t="inlineStr">
         <is>
-          <t>d8+2</t>
+          <t>d6+4</t>
         </is>
       </c>
       <c r="H25" s="36" t="inlineStr">
@@ -15646,7 +15646,7 @@
       </c>
       <c r="AJ25" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k6 kłute</t>
         </is>
       </c>
       <c r="AK25" s="43" t="n">
@@ -15689,12 +15689,12 @@
       </c>
       <c r="F26" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G26" s="36" t="inlineStr">
         <is>
-          <t>d10+2</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H26" s="36" t="inlineStr">
@@ -15746,7 +15746,7 @@
       </c>
       <c r="AJ26" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK26" s="43" t="n">
@@ -15789,12 +15789,12 @@
       </c>
       <c r="F27" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G27" s="36" t="inlineStr">
         <is>
-          <t>d10+3</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H27" s="36" t="inlineStr">
@@ -15846,7 +15846,7 @@
       </c>
       <c r="AJ27" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK27" s="43" t="n">
@@ -15892,12 +15892,12 @@
       </c>
       <c r="F28" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G28" s="36" t="inlineStr">
         <is>
-          <t>d8+3</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H28" s="36" t="inlineStr">
@@ -15949,7 +15949,7 @@
       </c>
       <c r="AJ28" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK28" s="41" t="inlineStr">
@@ -15997,12 +15997,12 @@
       </c>
       <c r="F29" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G29" s="36" t="inlineStr">
         <is>
-          <t>d10+3</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H29" s="36" t="inlineStr">
@@ -16054,7 +16054,7 @@
       </c>
       <c r="AJ29" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK29" s="43" t="n">
@@ -16100,12 +16100,12 @@
       </c>
       <c r="F30" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G30" s="36" t="inlineStr">
         <is>
-          <t>d8+3</t>
+          <t>d6+4</t>
         </is>
       </c>
       <c r="H30" s="36" t="inlineStr">
@@ -16157,7 +16157,7 @@
       </c>
       <c r="AJ30" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k6 kłute</t>
         </is>
       </c>
       <c r="AK30" s="43" t="n">
@@ -16207,12 +16207,12 @@
       </c>
       <c r="F31" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G31" s="36" t="inlineStr">
         <is>
-          <t>d8+2</t>
+          <t>d6+4</t>
         </is>
       </c>
       <c r="H31" s="36" t="inlineStr">
@@ -16264,7 +16264,7 @@
       </c>
       <c r="AJ31" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k6 kłute</t>
         </is>
       </c>
       <c r="AK31" s="43" t="n">
@@ -16310,12 +16310,12 @@
       </c>
       <c r="F32" s="38" t="inlineStr">
         <is>
-          <t>Very Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G32" s="36" t="inlineStr">
         <is>
-          <t>d8+1</t>
+          <t>d6+4</t>
         </is>
       </c>
       <c r="H32" s="36" t="inlineStr">
@@ -16367,7 +16367,7 @@
       </c>
       <c r="AJ32" s="41" t="inlineStr">
         <is>
-          <t>Śrut - patrz zasady śrutówek</t>
+          <t>3k4 kłute (breneka: 3k6 obuch.)</t>
         </is>
       </c>
       <c r="AK32" s="43" t="n">
@@ -16410,12 +16410,12 @@
       </c>
       <c r="F33" s="38" t="inlineStr">
         <is>
-          <t>Very Close</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="G33" s="36" t="inlineStr">
         <is>
-          <t>d8+1</t>
+          <t>d6+2</t>
         </is>
       </c>
       <c r="H33" s="36" t="inlineStr">
@@ -16467,7 +16467,7 @@
       </c>
       <c r="AJ33" s="41" t="inlineStr">
         <is>
-          <t>Śrut - patrz zasady śrutówek</t>
+          <t>2k4 kłute (breneka: 2k6 obuch.)</t>
         </is>
       </c>
       <c r="AK33" s="43" t="n">
@@ -16510,12 +16510,12 @@
       </c>
       <c r="F34" s="38" t="inlineStr">
         <is>
-          <t>Very Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G34" s="36" t="inlineStr">
         <is>
-          <t>d8+1</t>
+          <t>d6+7</t>
         </is>
       </c>
       <c r="H34" s="36" t="inlineStr">
@@ -16567,7 +16567,7 @@
       </c>
       <c r="AJ34" s="41" t="inlineStr">
         <is>
-          <t>Śrut - patrz zasady śrutówek</t>
+          <t>4k4 kłute (breneka: 4k6 obuch.)</t>
         </is>
       </c>
       <c r="AK34" s="43" t="n">
@@ -16813,12 +16813,12 @@
       </c>
       <c r="F37" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G37" s="36" t="inlineStr">
         <is>
-          <t>d10+4</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H37" s="36" t="inlineStr">
@@ -16873,7 +16873,7 @@
       </c>
       <c r="AJ37" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK37" s="43" t="n">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="G38" s="36" t="inlineStr">
         <is>
-          <t>d12+8</t>
+          <t>d12+4</t>
         </is>
       </c>
       <c r="H38" s="36" t="inlineStr">
@@ -16981,7 +16981,7 @@
       </c>
       <c r="AJ38" s="41" t="inlineStr">
         <is>
-          <t>Krytyczne</t>
+          <t>1k20 kłute</t>
         </is>
       </c>
       <c r="AK38" s="43" t="n">
@@ -17027,12 +17027,12 @@
       </c>
       <c r="F39" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G39" s="36" t="inlineStr">
         <is>
-          <t>d10+4</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H39" s="36" t="inlineStr">
@@ -17087,7 +17087,7 @@
       </c>
       <c r="AJ39" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK39" s="43" t="n">
@@ -17133,12 +17133,12 @@
       </c>
       <c r="F40" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G40" s="36" t="inlineStr">
         <is>
-          <t>d8+4</t>
+          <t>d6+4</t>
         </is>
       </c>
       <c r="H40" s="36" t="inlineStr">
@@ -17190,7 +17190,7 @@
       </c>
       <c r="AJ40" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k6 kłute</t>
         </is>
       </c>
       <c r="AK40" s="43" t="n">
@@ -17241,7 +17241,7 @@
       </c>
       <c r="G41" s="36" t="inlineStr">
         <is>
-          <t>d10+3</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H41" s="36" t="inlineStr">
@@ -17293,7 +17293,7 @@
       </c>
       <c r="AJ41" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK41" s="43" t="n">
@@ -17341,7 +17341,7 @@
       </c>
       <c r="G42" s="36" t="inlineStr">
         <is>
-          <t>d10+3</t>
+          <t>d8+5</t>
         </is>
       </c>
       <c r="H42" s="36" t="inlineStr">
@@ -17393,7 +17393,7 @@
       </c>
       <c r="AJ42" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>2k8 kłute</t>
         </is>
       </c>
       <c r="AK42" s="43" t="n">
@@ -17441,7 +17441,7 @@
       </c>
       <c r="G43" s="36" t="inlineStr">
         <is>
-          <t>d12+6</t>
+          <t>d12+15</t>
         </is>
       </c>
       <c r="H43" s="36" t="inlineStr">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="AJ43" s="41" t="inlineStr">
         <is>
-          <t>Krytyczne</t>
+          <t>2k20 kłute</t>
         </is>
       </c>
       <c r="AK43" s="43" t="n">
@@ -17539,7 +17539,7 @@
       </c>
       <c r="F44" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G44" s="36" t="inlineStr">
@@ -17596,7 +17596,7 @@
       </c>
       <c r="AJ44" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>6k6 wybuchowe</t>
         </is>
       </c>
       <c r="AK44" s="43" t="n">
@@ -17639,7 +17639,7 @@
       </c>
       <c r="F45" s="38" t="inlineStr">
         <is>
-          <t>Far</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G45" s="36" t="inlineStr">
@@ -17696,7 +17696,7 @@
       </c>
       <c r="AJ45" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>6k6 wybuchowe</t>
         </is>
       </c>
       <c r="AK45" s="43" t="n">
@@ -17796,7 +17796,7 @@
       </c>
       <c r="AJ46" s="41" t="inlineStr">
         <is>
-          <t>Krytyczne</t>
+          <t>15k6 wybuchowe</t>
         </is>
       </c>
       <c r="AK46" s="43" t="n">
@@ -17893,7 +17893,7 @@
       </c>
       <c r="AJ47" s="41" t="inlineStr">
         <is>
-          <t>Krytyczne</t>
+          <t>20k6 wybuchowe</t>
         </is>
       </c>
       <c r="AK47" s="43" t="n">
@@ -17993,7 +17993,7 @@
       </c>
       <c r="AJ48" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>10k6 cięte + 10k6 wybuchowe</t>
         </is>
       </c>
       <c r="AK48" s="43" t="n">
@@ -18033,7 +18033,7 @@
       </c>
       <c r="F49" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Very Far</t>
         </is>
       </c>
       <c r="G49" s="36" t="inlineStr">
@@ -18093,7 +18093,7 @@
       </c>
       <c r="AJ49" s="41" t="inlineStr">
         <is>
-          <t>Ciężkie</t>
+          <t>6k6 od ognia (linia 36 m)</t>
         </is>
       </c>
       <c r="AK49" s="43" t="n">
@@ -18321,7 +18321,7 @@
       </c>
       <c r="F52" s="38" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Far</t>
         </is>
       </c>
       <c r="G52" s="36" t="inlineStr">
@@ -30252,7 +30252,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
@@ -34611,7 +34611,7 @@
         <v>1</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB35" s="12" t="inlineStr">
         <is>

</xml_diff>